<commit_message>
file paths and corrected FF
</commit_message>
<xml_diff>
--- a/EQE/Plots/Boxplot output_results.xlsx
+++ b/EQE/Plots/Boxplot output_results.xlsx
@@ -418,28 +418,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se %</t>
+          <t>CdS1 %</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se %</t>
+          <t>CdS2 %</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se %</t>
+          <t>CdS31 %</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se %</t>
+          <t>CdS32 %</t>
         </is>
       </c>
     </row>
@@ -448,16 +448,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.934741554793868</v>
+        <v>0.7225835861726874</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4441288975489255</v>
+        <v>1.07173287471119</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2418793350126485</v>
+        <v>3.439230010020025</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1331462135605068</v>
+        <v>3.334850137961349</v>
       </c>
     </row>
     <row r="3">
@@ -465,16 +465,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.948624654779022</v>
+        <v>0.6870648845482235</v>
       </c>
       <c r="C3" t="n">
-        <v>0.495328743647059</v>
+        <v>1.694234371311958</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6675742033598158</v>
+        <v>3.691574518202918</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1184290133969196</v>
+        <v>3.350969570798699</v>
       </c>
     </row>
     <row r="4">
@@ -482,16 +482,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.6000584326916727</v>
+        <v>0.6212442906003888</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8965926537649891</v>
+        <v>1.222126253840952</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3857627116985633</v>
+        <v>3.259296403135965</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1105271609600943</v>
+        <v>2.941633670262369</v>
       </c>
     </row>
     <row r="5">
@@ -499,16 +499,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.143495594855657</v>
+        <v>0.6355627671927508</v>
       </c>
       <c r="C5" t="n">
-        <v>1.470398962784452</v>
+        <v>0.6326689363165827</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2645837702842248</v>
+        <v>3.73106090794139</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2545384216212359</v>
+        <v>3.137753436450121</v>
       </c>
     </row>
     <row r="6">
@@ -516,16 +516,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.539481531687119</v>
+        <v>0.8742040437321176</v>
       </c>
       <c r="C6" t="n">
-        <v>1.126613103994447</v>
+        <v>1.275251126356085</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1982251397949337</v>
+        <v>3.678796123856065</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8985393952225005</v>
+        <v>3.011973013552621</v>
       </c>
     </row>
     <row r="7">
@@ -533,16 +533,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.6489668698942753</v>
+        <v>0.2754919294747481</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2067477929121247</v>
+        <v>0.1597135322025925</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08714887449675331</v>
+        <v>4.566031125938888</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3530152576151716</v>
+        <v>2.860955094798665</v>
       </c>
     </row>
     <row r="8">
@@ -550,16 +550,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1102481469409318</v>
+        <v>0.2196609703587939</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2291544908874178</v>
+        <v>0.5658180201850996</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07396222356618901</v>
+        <v>4.205242946812436</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5148056862591703</v>
+        <v>2.950181854342782</v>
       </c>
     </row>
     <row r="9">
@@ -567,16 +567,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>0.3115077271178758</v>
+        <v>0.3547430324743331</v>
       </c>
       <c r="C9" t="n">
-        <v>1.517485502007893</v>
+        <v>0.9283719747181997</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1413842936466547</v>
+        <v>3.852973697250552</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2577979357514264</v>
+        <v>3.156396618873116</v>
       </c>
     </row>
     <row r="10">
@@ -584,16 +584,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.241856904554398</v>
+        <v>0.4504215349752327</v>
       </c>
       <c r="C10" t="n">
-        <v>1.972980115921098</v>
+        <v>1.176542232448382</v>
       </c>
       <c r="D10" t="n">
-        <v>0.4028309171369147</v>
+        <v>4.142962664455253</v>
       </c>
       <c r="E10" t="n">
-        <v>1.152188858444594</v>
+        <v>3.045270225827752</v>
       </c>
     </row>
     <row r="11">
@@ -601,16 +601,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.7045900090504822</v>
+        <v>0.4676259060745825</v>
       </c>
       <c r="C11" t="n">
-        <v>2.18719680815832</v>
+        <v>0.9016824454641856</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3098331248887014</v>
+        <v>3.945070233083724</v>
       </c>
       <c r="E11" t="n">
-        <v>1.130755083709705</v>
+        <v>2.756097370078937</v>
       </c>
     </row>
     <row r="12">
@@ -618,14 +618,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>2.086366784043495</v>
+        <v>0.2663902621834792</v>
       </c>
       <c r="C12" t="n">
-        <v>3.378107393299261</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>1.163239832153524</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.526438219243497</v>
+      </c>
       <c r="E12" t="n">
-        <v>1.196439232090816</v>
+        <v>2.748281887491131</v>
       </c>
     </row>
     <row r="13">
@@ -633,22 +635,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>2.879246049862312</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>0.2537367247297639</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.9810732039118404</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.35783969647746</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.640737590631845</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.287407990780198</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>0.2020126154891384</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.8566067960574061</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.232588407744345</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.788824703415374</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.09867539295046369</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.8901593471195953</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.740615923534082</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.741443340226801</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1588351938268994</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3094290820179671</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.561948644017728</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.75251527389286</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3064597974535775</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3576396920037894</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.627912787808238</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.666137909042214</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.2116692624932895</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.7514585236630202</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.205251550525309</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.795826073233617</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3023529475782489</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5623441449488629</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.215205186605834</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.122448116382334</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.3197793105627515</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.8732136142599037</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3.681328778591477</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2.613627635405393</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.3739453305400589</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.015642498945611</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3.437848561982528</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.35976198870998</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.3550760203020625</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.090288452192552</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3.044020750625925</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.449477215915834</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.3201122983904808</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.60128702657655</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3.484127071238697</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2.745676726628529</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.3005770124970257</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.36175909260481</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3.094328483324796</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.506546521062208</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.2138891813448185</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.480496255236553</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.426159512142258</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.175365446403936</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.32732703465795</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.334645920029303</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3.224529960858943</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.22934112302597</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -661,28 +879,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se V</t>
+          <t>CdS1 V</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se V</t>
+          <t>CdS2 V</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se V</t>
+          <t>CdS31 V</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se V</t>
+          <t>CdS32 V</t>
         </is>
       </c>
     </row>
@@ -691,16 +909,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.3242795</v>
+        <v>0.39583928</v>
       </c>
       <c r="C2" t="n">
-        <v>0.13526426</v>
+        <v>0.28590184</v>
       </c>
       <c r="D2" t="n">
-        <v>0.13766524</v>
+        <v>0.35526711</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06559524</v>
+        <v>0.37567141</v>
       </c>
     </row>
     <row r="3">
@@ -708,16 +926,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.33148791</v>
+        <v>0.38945222</v>
       </c>
       <c r="C3" t="n">
-        <v>0.14847342</v>
+        <v>0.33487447</v>
       </c>
       <c r="D3" t="n">
-        <v>0.27197523</v>
+        <v>0.35624521</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0696874</v>
+        <v>0.37535893</v>
       </c>
     </row>
     <row r="4">
@@ -725,16 +943,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.17293432</v>
+        <v>0.36128128</v>
       </c>
       <c r="C4" t="n">
-        <v>0.23489243</v>
+        <v>0.29911859</v>
       </c>
       <c r="D4" t="n">
-        <v>0.18035255</v>
+        <v>0.3485958</v>
       </c>
       <c r="E4" t="n">
-        <v>0.065423</v>
+        <v>0.37101022</v>
       </c>
     </row>
     <row r="5">
@@ -742,16 +960,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0.263739</v>
+        <v>0.36031146</v>
       </c>
       <c r="C5" t="n">
-        <v>0.26837173</v>
+        <v>0.21823373</v>
       </c>
       <c r="D5" t="n">
-        <v>0.14559311</v>
+        <v>0.36104157</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0887568</v>
+        <v>0.38065267</v>
       </c>
     </row>
     <row r="6">
@@ -759,16 +977,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.30209494</v>
+        <v>0.39466894</v>
       </c>
       <c r="C6" t="n">
-        <v>0.24815251</v>
+        <v>0.29939737</v>
       </c>
       <c r="D6" t="n">
-        <v>0.12967689</v>
+        <v>0.36317552</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2650255</v>
+        <v>0.37582084</v>
       </c>
     </row>
     <row r="7">
@@ -776,16 +994,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.15662631</v>
+        <v>0.38143188</v>
       </c>
       <c r="C7" t="n">
-        <v>0.09454997</v>
+        <v>0.07801342999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06916949999999999</v>
+        <v>0.38417545</v>
       </c>
       <c r="E7" t="n">
-        <v>0.12858896</v>
+        <v>0.37915835</v>
       </c>
     </row>
     <row r="8">
@@ -793,16 +1011,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.06911703</v>
+        <v>0.40273852</v>
       </c>
       <c r="C8" t="n">
-        <v>0.05278817</v>
+        <v>0.20242075</v>
       </c>
       <c r="D8" t="n">
-        <v>0.05074155</v>
+        <v>0.37325493</v>
       </c>
       <c r="E8" t="n">
-        <v>0.14656392</v>
+        <v>0.38243128</v>
       </c>
     </row>
     <row r="9">
@@ -810,16 +1028,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>0.07495999</v>
+        <v>0.36550189</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2802774</v>
+        <v>0.27454712</v>
       </c>
       <c r="D9" t="n">
-        <v>0.08671571</v>
+        <v>0.36952007</v>
       </c>
       <c r="E9" t="n">
-        <v>0.11050598</v>
+        <v>0.38236716</v>
       </c>
     </row>
     <row r="10">
@@ -827,16 +1045,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0.23712544</v>
+        <v>0.37661692</v>
       </c>
       <c r="C10" t="n">
-        <v>0.31310053</v>
+        <v>0.29808814</v>
       </c>
       <c r="D10" t="n">
-        <v>0.18391567</v>
+        <v>0.36464543</v>
       </c>
       <c r="E10" t="n">
-        <v>0.26156292</v>
+        <v>0.37184142</v>
       </c>
     </row>
     <row r="11">
@@ -844,16 +1062,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.18951907</v>
+        <v>0.40977589</v>
       </c>
       <c r="C11" t="n">
-        <v>0.33753093</v>
+        <v>0.27797018</v>
       </c>
       <c r="D11" t="n">
-        <v>0.14635379</v>
+        <v>0.36186303</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2729874</v>
+        <v>0.36069398</v>
       </c>
     </row>
     <row r="12">
@@ -861,14 +1079,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0.32984343</v>
+        <v>0.38712151</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3415921</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>0.28656075</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.32770751</v>
+      </c>
       <c r="E12" t="n">
-        <v>0.25275656</v>
+        <v>0.36163805</v>
       </c>
     </row>
     <row r="13">
@@ -876,22 +1096,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>0.33689226</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>0.25961971</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.25658739</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.36732332</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.3641843</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0.2375136</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>0.23891119</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.26016105</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.3684908</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.37403498</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.15666157</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.264496</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.37846602</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.38070717</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.36547692</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.13986286</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.3752776</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.37389124</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.26685594</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.14194758</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.3755534</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.36964348</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.19981049</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.24211232</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.33478432</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.37461582</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.28219999</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.17407841</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.36065483</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.38208378</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.36381487</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.24878627</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.36851292</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.36460307</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.30773187</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.26136434</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.36580805</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.37817283</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.30193057</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.2345453</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.35230196</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.38739785</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.3622594</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.26609076</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.36148494</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.34855739</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.28152101</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.28275494</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.35017888</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.38610293</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.20320389</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.17031921</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.36824807</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.38349557</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.26485068</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.31203721</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.35516014</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.3837273</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -904,28 +1340,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se mA/cm2</t>
+          <t>CdS1 mA/cm2</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se mA/cm2</t>
+          <t>CdS2 mA/cm2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se mA/cm2</t>
+          <t>CdS31 mA/cm2</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se mA/cm2</t>
+          <t>CdS32 mA/cm2</t>
         </is>
       </c>
     </row>
@@ -934,16 +1370,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>14.45286024895179</v>
+        <v>7.126938920875027</v>
       </c>
       <c r="C2" t="n">
-        <v>11.93737338386061</v>
+        <v>9.430307885742318</v>
       </c>
       <c r="D2" t="n">
-        <v>6.504377107432765</v>
+        <v>21.3802944403496</v>
       </c>
       <c r="E2" t="n">
-        <v>7.596721041907775</v>
+        <v>15.64603187108552</v>
       </c>
     </row>
     <row r="3">
@@ -951,16 +1387,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>13.94387211202528</v>
+        <v>6.939840608198002</v>
       </c>
       <c r="C3" t="n">
-        <v>12.20064063275801</v>
+        <v>13.39495906546591</v>
       </c>
       <c r="D3" t="n">
-        <v>8.137738998251317</v>
+        <v>21.14810601883022</v>
       </c>
       <c r="E3" t="n">
-        <v>6.370107964016063</v>
+        <v>15.71121416819021</v>
       </c>
     </row>
     <row r="4">
@@ -968,16 +1404,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>10.733455019992</v>
+        <v>7.040978013250347</v>
       </c>
       <c r="C4" t="n">
-        <v>13.58397123721938</v>
+        <v>11.88795001340611</v>
       </c>
       <c r="D4" t="n">
-        <v>7.676114467430839</v>
+        <v>20.97415990705442</v>
       </c>
       <c r="E4" t="n">
-        <v>6.276745868699383</v>
+        <v>15.13347386351254</v>
       </c>
     </row>
     <row r="5">
@@ -985,16 +1421,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>12.52059470420762</v>
+        <v>7.275563120661765</v>
       </c>
       <c r="C5" t="n">
-        <v>17.9724163969221</v>
+        <v>9.590541338447643</v>
       </c>
       <c r="D5" t="n">
-        <v>6.650289090848409</v>
+        <v>20.55980595364126</v>
       </c>
       <c r="E5" t="n">
-        <v>10.61138718721289</v>
+        <v>14.90180847654381</v>
       </c>
     </row>
     <row r="6">
@@ -1002,16 +1438,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>13.33773583963854</v>
+        <v>8.937341394552979</v>
       </c>
       <c r="C6" t="n">
-        <v>15.28382458343588</v>
+        <v>10.40757818759585</v>
       </c>
       <c r="D6" t="n">
-        <v>5.735213700345992</v>
+        <v>20.70364691662024</v>
       </c>
       <c r="E6" t="n">
-        <v>11.25114191273823</v>
+        <v>14.80235319602177</v>
       </c>
     </row>
     <row r="7">
@@ -1019,16 +1455,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>13.89767077950664</v>
+        <v>3.301776635340624</v>
       </c>
       <c r="C7" t="n">
-        <v>8.035858807509911</v>
+        <v>7.771317944406994</v>
       </c>
       <c r="D7" t="n">
-        <v>4.725712780820636</v>
+        <v>20.31502635852031</v>
       </c>
       <c r="E7" t="n">
-        <v>10.174612313522</v>
+        <v>14.10064178523019</v>
       </c>
     </row>
     <row r="8">
@@ -1036,16 +1472,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>6.012948488728604</v>
+        <v>2.550987836901052</v>
       </c>
       <c r="C8" t="n">
-        <v>16.29220550904066</v>
+        <v>9.130108398800781</v>
       </c>
       <c r="D8" t="n">
-        <v>5.510821353282699</v>
+        <v>20.68065924137806</v>
       </c>
       <c r="E8" t="n">
-        <v>12.40267241846973</v>
+        <v>14.4240644466058</v>
       </c>
     </row>
     <row r="9">
@@ -1053,16 +1489,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>13.76973541800188</v>
+        <v>4.178541521961894</v>
       </c>
       <c r="C9" t="n">
-        <v>17.6072160671954</v>
+        <v>9.536237475041665</v>
       </c>
       <c r="D9" t="n">
-        <v>6.135320920050396</v>
+        <v>21.2255276278662</v>
       </c>
       <c r="E9" t="n">
-        <v>8.521968244010232</v>
+        <v>14.9825084794556</v>
       </c>
     </row>
     <row r="10">
@@ -1070,16 +1506,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>14.0383833295848</v>
+        <v>5.068651717149392</v>
       </c>
       <c r="C10" t="n">
-        <v>17.44617089140872</v>
+        <v>10.66237400657964</v>
       </c>
       <c r="D10" t="n">
-        <v>7.961264292705112</v>
+        <v>21.7630071553327</v>
       </c>
       <c r="E10" t="n">
-        <v>13.8616408698451</v>
+        <v>15.23807370987138</v>
       </c>
     </row>
     <row r="11">
@@ -1087,16 +1523,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>12.12630414795415</v>
+        <v>4.569860126127121</v>
       </c>
       <c r="C11" t="n">
-        <v>17.29559824904748</v>
+        <v>8.530784919745106</v>
       </c>
       <c r="D11" t="n">
-        <v>7.885888151761685</v>
+        <v>21.94411275970764</v>
       </c>
       <c r="E11" t="n">
-        <v>12.86157602494002</v>
+        <v>15.16494860294173</v>
       </c>
     </row>
     <row r="12">
@@ -1104,14 +1540,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>14.25587336066282</v>
+        <v>2.92733460905713</v>
       </c>
       <c r="C12" t="n">
-        <v>21.42174449723805</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>11.71357055945984</v>
+      </c>
+      <c r="D12" t="n">
+        <v>20.65527281976359</v>
+      </c>
       <c r="E12" t="n">
-        <v>14.23632039923074</v>
+        <v>17.27686388179589</v>
       </c>
     </row>
     <row r="13">
@@ -1119,22 +1557,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>15.77471700182574</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>4.036361069525894</v>
+      </c>
+      <c r="C13" t="n">
+        <v>11.49972264659846</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21.60992773557883</v>
+      </c>
+      <c r="E13" t="n">
+        <v>14.94230882834599</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>15.38058888691601</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>3.483910499091599</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9.329645123417292</v>
+      </c>
+      <c r="D14" t="n">
+        <v>20.8709763527791</v>
+      </c>
+      <c r="E14" t="n">
+        <v>14.80831079999928</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2.526423347048647</v>
+      </c>
+      <c r="C15" t="n">
+        <v>9.877356695824744</v>
+      </c>
+      <c r="D15" t="n">
+        <v>20.72036487843216</v>
+      </c>
+      <c r="E15" t="n">
+        <v>14.42699127156478</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2.030146158213153</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8.197378913606373</v>
+      </c>
+      <c r="D16" t="n">
+        <v>20.87499124369842</v>
+      </c>
+      <c r="E16" t="n">
+        <v>14.30734245296704</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4.892954508108426</v>
+      </c>
+      <c r="C17" t="n">
+        <v>9.17594181901671</v>
+      </c>
+      <c r="D17" t="n">
+        <v>20.43541687267661</v>
+      </c>
+      <c r="E17" t="n">
+        <v>14.08833649514162</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>4.364951437803061</v>
+      </c>
+      <c r="C18" t="n">
+        <v>9.383842864171241</v>
+      </c>
+      <c r="D18" t="n">
+        <v>18.99187957254924</v>
+      </c>
+      <c r="E18" t="n">
+        <v>14.33949344330939</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>4.540174971659082</v>
+      </c>
+      <c r="C19" t="n">
+        <v>11.53720647211824</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21.65571018986886</v>
+      </c>
+      <c r="E19" t="n">
+        <v>14.67976025256869</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3.873173658193006</v>
+      </c>
+      <c r="C20" t="n">
+        <v>11.19396745877454</v>
+      </c>
+      <c r="D20" t="n">
+        <v>22.90148535219879</v>
+      </c>
+      <c r="E20" t="n">
+        <v>14.4519979745922</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>5.115867659584711</v>
+      </c>
+      <c r="C21" t="n">
+        <v>10.68812651306232</v>
+      </c>
+      <c r="D21" t="n">
+        <v>21.91316260217041</v>
+      </c>
+      <c r="E21" t="n">
+        <v>18.50008056232052</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4.968804340240453</v>
+      </c>
+      <c r="C22" t="n">
+        <v>16.21039284599291</v>
+      </c>
+      <c r="D22" t="n">
+        <v>20.98034596229393</v>
+      </c>
+      <c r="E22" t="n">
+        <v>14.97461176469565</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3.920356490538654</v>
+      </c>
+      <c r="C23" t="n">
+        <v>19.60314768130189</v>
+      </c>
+      <c r="D23" t="n">
+        <v>21.61360229526204</v>
+      </c>
+      <c r="E23" t="n">
+        <v>15.30459065530936</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4.539079563801389</v>
+      </c>
+      <c r="C24" t="n">
+        <v>14.92484758514928</v>
+      </c>
+      <c r="D24" t="n">
+        <v>21.60311119896707</v>
+      </c>
+      <c r="E24" t="n">
+        <v>16.31440446843945</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4.352424502321449</v>
+      </c>
+      <c r="C25" t="n">
+        <v>9.907511602029963</v>
+      </c>
+      <c r="D25" t="n">
+        <v>22.29578218453164</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15.27503378646046</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>5.255182418775272</v>
+      </c>
+      <c r="C26" t="n">
+        <v>9.962153642953758</v>
+      </c>
+      <c r="D26" t="n">
+        <v>21.43848871023768</v>
+      </c>
+      <c r="E26" t="n">
+        <v>14.42479045609144</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1147,28 +1801,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se %</t>
+          <t>CdS1 %</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se %</t>
+          <t>CdS2 %</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se %</t>
+          <t>CdS31 %</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se %</t>
+          <t>CdS32 %</t>
         </is>
       </c>
     </row>
@@ -1177,16 +1831,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>43.08390781883061</v>
+        <v>24.9718</v>
       </c>
       <c r="C2" t="n">
-        <v>24.06570261243263</v>
+        <v>38.7567</v>
       </c>
       <c r="D2" t="n">
-        <v>48.10710493061145</v>
+        <v>44.1464</v>
       </c>
       <c r="E2" t="n">
-        <v>25.60979233893447</v>
+        <v>54.5811</v>
       </c>
     </row>
     <row r="3">
@@ -1194,16 +1848,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>43.99773542315287</v>
+        <v>24.7854</v>
       </c>
       <c r="C3" t="n">
-        <v>23.92176975791046</v>
+        <v>36.8263</v>
       </c>
       <c r="D3" t="n">
-        <v>53.7179549022679</v>
+        <v>47.7744</v>
       </c>
       <c r="E3" t="n">
-        <v>25.58063461904004</v>
+        <v>54.662</v>
       </c>
     </row>
     <row r="4">
@@ -1211,16 +1865,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>33.73855482571398</v>
+        <v>23.8115</v>
       </c>
       <c r="C4" t="n">
-        <v>24.58230885279717</v>
+        <v>33.5106</v>
       </c>
       <c r="D4" t="n">
-        <v>49.62933526079136</v>
+        <v>43.4638</v>
       </c>
       <c r="E4" t="n">
-        <v>25.7950653507636</v>
+        <v>50.4007</v>
       </c>
     </row>
     <row r="5">
@@ -1228,16 +1882,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>36.14126459771517</v>
+        <v>23.6388</v>
       </c>
       <c r="C5" t="n">
-        <v>26.66979715881957</v>
+        <v>29.4711</v>
       </c>
       <c r="D5" t="n">
-        <v>48.66397718260832</v>
+        <v>49.0077</v>
       </c>
       <c r="E5" t="n">
-        <v>25.90774778910557</v>
+        <v>53.2142</v>
       </c>
     </row>
     <row r="6">
@@ -1245,16 +1899,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>39.87493143404341</v>
+        <v>24.1649</v>
       </c>
       <c r="C6" t="n">
-        <v>25.9887490179098</v>
+        <v>39.9017</v>
       </c>
       <c r="D6" t="n">
-        <v>47.46390901645093</v>
+        <v>47.7031</v>
       </c>
       <c r="E6" t="n">
-        <v>28.88963085872495</v>
+        <v>52.0853</v>
       </c>
     </row>
     <row r="7">
@@ -1262,16 +1916,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>31.11400050866929</v>
+        <v>21.3291</v>
       </c>
       <c r="C7" t="n">
-        <v>23.80601374589745</v>
+        <v>25.6907</v>
       </c>
       <c r="D7" t="n">
-        <v>47.46955108587339</v>
+        <v>57.0428</v>
       </c>
       <c r="E7" t="n">
-        <v>25.86593480884031</v>
+        <v>51.4792</v>
       </c>
     </row>
     <row r="8">
@@ -1279,16 +1933,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>27.69155522981886</v>
+        <v>20.8455</v>
       </c>
       <c r="C8" t="n">
-        <v>23.30963940228538</v>
+        <v>29.8488</v>
       </c>
       <c r="D8" t="n">
-        <v>47.10131202156744</v>
+        <v>53.1156</v>
       </c>
       <c r="E8" t="n">
-        <v>27.1523167150157</v>
+        <v>51.4504</v>
       </c>
     </row>
     <row r="9">
@@ -1296,16 +1950,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>31.49454159860232</v>
+        <v>22.648</v>
       </c>
       <c r="C9" t="n">
-        <v>26.90232539683772</v>
+        <v>34.573</v>
       </c>
       <c r="D9" t="n">
-        <v>47.32304534987016</v>
+        <v>47.8972</v>
       </c>
       <c r="E9" t="n">
-        <v>26.24194790497879</v>
+        <v>53.0028</v>
       </c>
     </row>
     <row r="10">
@@ -1313,16 +1967,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>38.93432378777104</v>
+        <v>23.0066</v>
       </c>
       <c r="C10" t="n">
-        <v>31.59926646847831</v>
+        <v>36.0911</v>
       </c>
       <c r="D10" t="n">
-        <v>48.9976115544565</v>
+        <v>50.9012</v>
       </c>
       <c r="E10" t="n">
-        <v>30.46860238467421</v>
+        <v>51.7024</v>
       </c>
     </row>
     <row r="11">
@@ -1330,16 +1984,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>31.99840312862661</v>
+        <v>24.3484</v>
       </c>
       <c r="C11" t="n">
-        <v>32.77844423171383</v>
+        <v>37.0754</v>
       </c>
       <c r="D11" t="n">
-        <v>47.81352925166274</v>
+        <v>48.4396</v>
       </c>
       <c r="E11" t="n">
-        <v>30.87812661027467</v>
+        <v>48.4722</v>
       </c>
     </row>
     <row r="12">
@@ -1347,14 +2001,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>46.30743138689935</v>
+        <v>22.9213</v>
       </c>
       <c r="C12" t="n">
-        <v>40.3885012864401</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>33.7879</v>
+      </c>
+      <c r="D12" t="n">
+        <v>36.3912</v>
+      </c>
       <c r="E12" t="n">
-        <v>31.87809466373715</v>
+        <v>42.3157</v>
       </c>
     </row>
     <row r="13">
@@ -1362,22 +2018,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>56.54368915007642</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>23.6069</v>
+      </c>
+      <c r="C13" t="n">
+        <v>32.4184</v>
+      </c>
+      <c r="D13" t="n">
+        <v>41.2446</v>
+      </c>
+      <c r="E13" t="n">
+        <v>46.6831</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>36.77957736715975</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>23.6656</v>
+      </c>
+      <c r="C14" t="n">
+        <v>34.4096</v>
+      </c>
+      <c r="D14" t="n">
+        <v>40.9806</v>
+      </c>
+      <c r="E14" t="n">
+        <v>48.4368</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>24.3011</v>
+      </c>
+      <c r="C15" t="n">
+        <v>33.2216</v>
+      </c>
+      <c r="D15" t="n">
+        <v>46.5083</v>
+      </c>
+      <c r="E15" t="n">
+        <v>48.0159</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>20.8705</v>
+      </c>
+      <c r="C16" t="n">
+        <v>26.3152</v>
+      </c>
+      <c r="D16" t="n">
+        <v>44.3315</v>
+      </c>
+      <c r="E16" t="n">
+        <v>49.4996</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>22.8871</v>
+      </c>
+      <c r="C17" t="n">
+        <v>26.7715</v>
+      </c>
+      <c r="D17" t="n">
+        <v>46.0893</v>
+      </c>
+      <c r="E17" t="n">
+        <v>49.251</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>23.6602</v>
+      </c>
+      <c r="C18" t="n">
+        <v>32.2487</v>
+      </c>
+      <c r="D18" t="n">
+        <v>33.8173</v>
+      </c>
+      <c r="E18" t="n">
+        <v>50.0689</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>23.0095</v>
+      </c>
+      <c r="C19" t="n">
+        <v>27.3004</v>
+      </c>
+      <c r="D19" t="n">
+        <v>40.1373</v>
+      </c>
+      <c r="E19" t="n">
+        <v>53.5535</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>22.128</v>
+      </c>
+      <c r="C20" t="n">
+        <v>30.5726</v>
+      </c>
+      <c r="D20" t="n">
+        <v>42.5296</v>
+      </c>
+      <c r="E20" t="n">
+        <v>47.717</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>23.1559</v>
+      </c>
+      <c r="C21" t="n">
+        <v>35.449</v>
+      </c>
+      <c r="D21" t="n">
+        <v>41.815</v>
+      </c>
+      <c r="E21" t="n">
+        <v>46.1979</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>23.0783</v>
+      </c>
+      <c r="C22" t="n">
+        <v>27.9602</v>
+      </c>
+      <c r="D22" t="n">
+        <v>40.1538</v>
+      </c>
+      <c r="E22" t="n">
+        <v>57.2032</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>21.977</v>
+      </c>
+      <c r="C23" t="n">
+        <v>29.9301</v>
+      </c>
+      <c r="D23" t="n">
+        <v>43.4796</v>
+      </c>
+      <c r="E23" t="n">
+        <v>49.5146</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>22.9301</v>
+      </c>
+      <c r="C24" t="n">
+        <v>31.4617</v>
+      </c>
+      <c r="D24" t="n">
+        <v>39.8812</v>
+      </c>
+      <c r="E24" t="n">
+        <v>53.5524</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>23.5756</v>
+      </c>
+      <c r="C25" t="n">
+        <v>27.7617</v>
+      </c>
+      <c r="D25" t="n">
+        <v>52.5614</v>
+      </c>
+      <c r="E25" t="n">
+        <v>52.1466</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>22.9319</v>
+      </c>
+      <c r="C26" t="n">
+        <v>41.8608</v>
+      </c>
+      <c r="D26" t="n">
+        <v>41.291</v>
+      </c>
+      <c r="E26" t="n">
+        <v>56.1257</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1390,28 +2262,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se Ohm cm$^2$</t>
+          <t>CdS1 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se Ohm cm$^2$</t>
+          <t>CdS2 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se Ohm cm$^2$</t>
+          <t>CdS31 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se Ohm cm$^2$</t>
+          <t>CdS32 Ohm cm$^2$</t>
         </is>
       </c>
     </row>
@@ -1420,16 +2292,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>9.324108183433355</v>
+        <v>50.31773125721282</v>
       </c>
       <c r="C2" t="n">
-        <v>10.26777981896216</v>
+        <v>13.37460563909487</v>
       </c>
       <c r="D2" t="n">
-        <v>20.07292592137726</v>
+        <v>6.042479974596063</v>
       </c>
       <c r="E2" t="n">
-        <v>8.372663763700194</v>
+        <v>5.462649089169353</v>
       </c>
     </row>
     <row r="3">
@@ -1437,16 +2309,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>9.378826234688209</v>
+        <v>50.14913790043208</v>
       </c>
       <c r="C3" t="n">
-        <v>11.15533709505658</v>
+        <v>11.62503022454319</v>
       </c>
       <c r="D3" t="n">
-        <v>23.34893484270998</v>
+        <v>5.395422702336701</v>
       </c>
       <c r="E3" t="n">
-        <v>10.66125851705404</v>
+        <v>5.61861983917749</v>
       </c>
     </row>
     <row r="4">
@@ -1454,16 +2326,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>10.498285164459</v>
+        <v>52.98103497810288</v>
       </c>
       <c r="C4" t="n">
-        <v>14.25975206021645</v>
+        <v>13.94425060085733</v>
       </c>
       <c r="D4" t="n">
-        <v>20.5276583968945</v>
+        <v>6.02912084221252</v>
       </c>
       <c r="E4" t="n">
-        <v>9.975156512797268</v>
+        <v>6.778294969595367</v>
       </c>
     </row>
     <row r="5">
@@ -1471,16 +2343,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>12.87200413644884</v>
+        <v>53.99936453510902</v>
       </c>
       <c r="C5" t="n">
-        <v>10.82922233176065</v>
+        <v>15.90129217228154</v>
       </c>
       <c r="D5" t="n">
-        <v>20.07024983585972</v>
+        <v>4.516255436824059</v>
       </c>
       <c r="E5" t="n">
-        <v>7.853095093718603</v>
+        <v>5.941586009115403</v>
       </c>
     </row>
     <row r="6">
@@ -1488,16 +2360,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>11.29680811816508</v>
+        <v>48.37112716075483</v>
       </c>
       <c r="C6" t="n">
-        <v>12.46043115066997</v>
+        <v>12.29002573329954</v>
       </c>
       <c r="D6" t="n">
-        <v>21.74703914767739</v>
+        <v>4.933382749288774</v>
       </c>
       <c r="E6" t="n">
-        <v>16.81960782964153</v>
+        <v>5.967090657367131</v>
       </c>
     </row>
     <row r="7">
@@ -1505,16 +2377,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>8.755618441329895</v>
+        <v>120.8562927047164</v>
       </c>
       <c r="C7" t="n">
-        <v>11.03433110829836</v>
+        <v>9.280419539422581</v>
       </c>
       <c r="D7" t="n">
-        <v>14.21822336093223</v>
+        <v>3.485610415784251</v>
       </c>
       <c r="E7" t="n">
-        <v>11.9940353811483</v>
+        <v>6.574395078435551</v>
       </c>
     </row>
     <row r="8">
@@ -1522,16 +2394,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>11.29379522324477</v>
+        <v>147.059410296244</v>
       </c>
       <c r="C8" t="n">
-        <v>3.18197892744066</v>
+        <v>15.12476056503753</v>
       </c>
       <c r="D8" t="n">
-        <v>9.005991145114157</v>
+        <v>3.855714659760845</v>
       </c>
       <c r="E8" t="n">
-        <v>10.08042711235501</v>
+        <v>7.27719057016556</v>
       </c>
     </row>
     <row r="9">
@@ -1539,16 +2411,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>4.120923795559327</v>
+        <v>87.74958359122506</v>
       </c>
       <c r="C9" t="n">
-        <v>10.50047809075473</v>
+        <v>15.22057486751145</v>
       </c>
       <c r="D9" t="n">
-        <v>14.00095940568573</v>
+        <v>5.458424380053783</v>
       </c>
       <c r="E9" t="n">
-        <v>11.88559376474818</v>
+        <v>6.598207066902462</v>
       </c>
     </row>
     <row r="10">
@@ -1556,16 +2428,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>8.707259156216191</v>
+        <v>73.88190560059991</v>
       </c>
       <c r="C10" t="n">
-        <v>9.223224318325306</v>
+        <v>13.64924528971436</v>
       </c>
       <c r="D10" t="n">
-        <v>20.90035641079593</v>
+        <v>4.565649566184273</v>
       </c>
       <c r="E10" t="n">
-        <v>12.73569167182101</v>
+        <v>6.06016399662628</v>
       </c>
     </row>
     <row r="11">
@@ -1573,16 +2445,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>11.21832368140057</v>
+        <v>69.84927642846648</v>
       </c>
       <c r="C11" t="n">
-        <v>8.930827200828212</v>
+        <v>15.09108053792624</v>
       </c>
       <c r="D11" t="n">
-        <v>17.8704233159873</v>
+        <v>4.91800361470608</v>
       </c>
       <c r="E11" t="n">
-        <v>13.0934393739958</v>
+        <v>6.493681575677569</v>
       </c>
     </row>
     <row r="12">
@@ -1590,14 +2462,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>8.751496600619307</v>
+        <v>113.8937896462192</v>
       </c>
       <c r="C12" t="n">
-        <v>5.567792489109745</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>13.23240184363969</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8.09836050519349</v>
+      </c>
       <c r="E12" t="n">
-        <v>9.821785659043996</v>
+        <v>7.414534795399701</v>
       </c>
     </row>
     <row r="13">
@@ -1605,22 +2479,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>4.375147138866716</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>71.78516768688978</v>
+      </c>
+      <c r="C13" t="n">
+        <v>13.32635299289849</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7.179635209420761</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7.496246475072278</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>9.124896975851817</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>76.44745126447278</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15.28057087962011</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7.629926970526018</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7.967657238337793</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>64.49375766085043</v>
+      </c>
+      <c r="C15" t="n">
+        <v>15.18006850642345</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5.792274128440994</v>
+      </c>
+      <c r="E15" t="n">
+        <v>8.361819866386151</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>186.3318162347515</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15.10453412357968</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6.089582888025115</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7.473298599083749</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>63.9172556327903</v>
+      </c>
+      <c r="C17" t="n">
+        <v>13.02497400680199</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5.792658286155887</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6.501944115006686</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>51.34295138432223</v>
+      </c>
+      <c r="C18" t="n">
+        <v>15.2469656834728</v>
+      </c>
+      <c r="D18" t="n">
+        <v>8.205597239824536</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7.205911489900778</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>69.61013077141411</v>
+      </c>
+      <c r="C19" t="n">
+        <v>12.38185282095869</v>
+      </c>
+      <c r="D19" t="n">
+        <v>7.43889809951024</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6.426503438619327</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>86.28525353813515</v>
+      </c>
+      <c r="C20" t="n">
+        <v>14.22980078123329</v>
+      </c>
+      <c r="D20" t="n">
+        <v>6.619310039237063</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.701114143460344</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>66.25735524568201</v>
+      </c>
+      <c r="C21" t="n">
+        <v>12.3639141546948</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6.987236265022505</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5.618325168341999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>66.83343195168955</v>
+      </c>
+      <c r="C22" t="n">
+        <v>11.34768353367829</v>
+      </c>
+      <c r="D22" t="n">
+        <v>6.405490369461297</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5.051321494797189</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>84.35976969349777</v>
+      </c>
+      <c r="C23" t="n">
+        <v>9.472041103692202</v>
+      </c>
+      <c r="D23" t="n">
+        <v>6.059052314554596</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6.039974860153582</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>69.83347956847352</v>
+      </c>
+      <c r="C24" t="n">
+        <v>11.82407529449587</v>
+      </c>
+      <c r="D24" t="n">
+        <v>6.515970212616899</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5.70673396966329</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>52.77456091442748</v>
+      </c>
+      <c r="C25" t="n">
+        <v>13.24478446452019</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3.932963880030928</v>
+      </c>
+      <c r="E25" t="n">
+        <v>6.575015950751788</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>59.06764410280962</v>
+      </c>
+      <c r="C26" t="n">
+        <v>11.43486810097261</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5.326209785509366</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5.538480977108592</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1633,28 +2723,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mo200Sb25Se Ohm cm$^2$</t>
+          <t>CdS1 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mo300Sb35Se Ohm cm$^2$</t>
+          <t>CdS2 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mo400deg400Sb35Se Ohm cm$^2$</t>
+          <t>CdS31 Ohm cm$^2$</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Mo400Sb30Se Ohm cm$^2$</t>
+          <t>CdS32 Ohm cm$^2$</t>
         </is>
       </c>
     </row>
@@ -1663,16 +2753,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>66.41528291672351</v>
+        <v>58.16303591796542</v>
       </c>
       <c r="C2" t="n">
-        <v>12.11531454696171</v>
+        <v>81.71178685427871</v>
       </c>
       <c r="D2" t="n">
-        <v>22.0138081840883</v>
+        <v>94.19213161860789</v>
       </c>
       <c r="E2" t="n">
-        <v>8.784094057406895</v>
+        <v>245.6066255368933</v>
       </c>
     </row>
     <row r="3">
@@ -1680,16 +2770,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>93.99360883908999</v>
+        <v>59.69672374616301</v>
       </c>
       <c r="C3" t="n">
-        <v>13.03332436274324</v>
+        <v>52.18484887140539</v>
       </c>
       <c r="D3" t="n">
-        <v>41.30229150532164</v>
+        <v>123.9929805976566</v>
       </c>
       <c r="E3" t="n">
-        <v>11.0672509788285</v>
+        <v>243.1309164987352</v>
       </c>
     </row>
     <row r="4">
@@ -1697,16 +2787,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>23.80113454094396</v>
+        <v>48.99138618397147</v>
       </c>
       <c r="C4" t="n">
-        <v>19.22040191197024</v>
+        <v>46.10473213480162</v>
       </c>
       <c r="D4" t="n">
-        <v>25.67226748847014</v>
+        <v>83.16959006369008</v>
       </c>
       <c r="E4" t="n">
-        <v>10.63183095284817</v>
+        <v>192.0803122103064</v>
       </c>
     </row>
     <row r="5">
@@ -1714,16 +2804,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>46.19441935977939</v>
+        <v>47.27310304452644</v>
       </c>
       <c r="C5" t="n">
-        <v>19.9574491586689</v>
+        <v>30.13073962170874</v>
       </c>
       <c r="D5" t="n">
-        <v>23.33272955810772</v>
+        <v>109.2852639702109</v>
       </c>
       <c r="E5" t="n">
-        <v>8.558983438983798</v>
+        <v>205.9252583926456</v>
       </c>
     </row>
     <row r="6">
@@ -1731,16 +2821,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>64.5804804470729</v>
+        <v>46.59897182106366</v>
       </c>
       <c r="C6" t="n">
-        <v>20.5471641790724</v>
+        <v>95.22117783569838</v>
       </c>
       <c r="D6" t="n">
-        <v>22.9840296399152</v>
+        <v>101.7623730396351</v>
       </c>
       <c r="E6" t="n">
-        <v>29.73729192511557</v>
+        <v>198.7523996414761</v>
       </c>
     </row>
     <row r="7">
@@ -1748,16 +2838,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>14.34745737998252</v>
+        <v>90.12288466003456</v>
       </c>
       <c r="C7" t="n">
-        <v>12.42630912164354</v>
+        <v>10.41582310993411</v>
       </c>
       <c r="D7" t="n">
-        <v>14.56923399564795</v>
+        <v>163.266437096643</v>
       </c>
       <c r="E7" t="n">
-        <v>13.19438630222652</v>
+        <v>208.8445162350408</v>
       </c>
     </row>
     <row r="8">
@@ -1765,16 +2855,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>11.58939794854865</v>
+        <v>117.1525748249155</v>
       </c>
       <c r="C8" t="n">
-        <v>3.304504351490356</v>
+        <v>30.16183516793411</v>
       </c>
       <c r="D8" t="n">
-        <v>9.143530374103769</v>
+        <v>134.362541670835</v>
       </c>
       <c r="E8" t="n">
-        <v>13.43883989323044</v>
+        <v>214.622585866113</v>
       </c>
     </row>
     <row r="9">
@@ -1782,16 +2872,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>6.969692930666804</v>
+        <v>73.55430251790206</v>
       </c>
       <c r="C9" t="n">
-        <v>21.06593245999063</v>
+        <v>56.45672316037282</v>
       </c>
       <c r="D9" t="n">
-        <v>14.18399790557088</v>
+        <v>108.298769335285</v>
       </c>
       <c r="E9" t="n">
-        <v>13.91061784973458</v>
+        <v>225.3264973271463</v>
       </c>
     </row>
     <row r="10">
@@ -1799,16 +2889,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>40.21344994265066</v>
+        <v>64.72178314995698</v>
       </c>
       <c r="C10" t="n">
-        <v>33.07152672017713</v>
+        <v>58.46183206247895</v>
       </c>
       <c r="D10" t="n">
-        <v>24.58395903014264</v>
+        <v>136.1386563636732</v>
       </c>
       <c r="E10" t="n">
-        <v>27.1556174795204</v>
+        <v>207.1909198873831</v>
       </c>
     </row>
     <row r="11">
@@ -1816,16 +2906,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>20.39232771938346</v>
+        <v>91.00252903417457</v>
       </c>
       <c r="C11" t="n">
-        <v>42.18073420502689</v>
+        <v>73.41062304249395</v>
       </c>
       <c r="D11" t="n">
-        <v>19.19957384713559</v>
+        <v>104.4852729142897</v>
       </c>
       <c r="E11" t="n">
-        <v>30.32653930075564</v>
+        <v>181.5203474139053</v>
       </c>
     </row>
     <row r="12">
@@ -1833,14 +2923,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>112.0406611605686</v>
+        <v>115.709419829221</v>
       </c>
       <c r="C12" t="n">
-        <v>95.96732535508755</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>42.00694255455875</v>
+      </c>
+      <c r="D12" t="n">
+        <v>37.6912056627539</v>
+      </c>
       <c r="E12" t="n">
-        <v>26.2456947527108</v>
+        <v>77.79215463786437</v>
       </c>
     </row>
     <row r="13">
@@ -1848,22 +2940,238 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>120.925375802889</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+        <v>58.17703057412109</v>
+      </c>
+      <c r="C13" t="n">
+        <v>36.30439404236335</v>
+      </c>
+      <c r="D13" t="n">
+        <v>90.78120853546915</v>
+      </c>
+      <c r="E13" t="n">
+        <v>162.097225672059</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>32.73375247603738</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+        <v>62.45369641003494</v>
+      </c>
+      <c r="C14" t="n">
+        <v>55.31507428237231</v>
+      </c>
+      <c r="D14" t="n">
+        <v>85.07867209209681</v>
+      </c>
+      <c r="E14" t="n">
+        <v>184.9480400100822</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>58.29674552843819</v>
+      </c>
+      <c r="C15" t="n">
+        <v>45.98477649308729</v>
+      </c>
+      <c r="D15" t="n">
+        <v>114.1499027105438</v>
+      </c>
+      <c r="E15" t="n">
+        <v>190.4052100152174</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>132.693761082258</v>
+      </c>
+      <c r="C16" t="n">
+        <v>18.71994191524921</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95.96306448294769</v>
+      </c>
+      <c r="E16" t="n">
+        <v>189.9306090619554</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>47.00196576708163</v>
+      </c>
+      <c r="C17" t="n">
+        <v>17.18906559685465</v>
+      </c>
+      <c r="D17" t="n">
+        <v>92.31563081653479</v>
+      </c>
+      <c r="E17" t="n">
+        <v>172.1487806311528</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>42.32023924714612</v>
+      </c>
+      <c r="C18" t="n">
+        <v>41.68618586459544</v>
+      </c>
+      <c r="D18" t="n">
+        <v>28.12217947200841</v>
+      </c>
+      <c r="E18" t="n">
+        <v>198.0174682408226</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>52.03130032093804</v>
+      </c>
+      <c r="C19" t="n">
+        <v>17.70422669071799</v>
+      </c>
+      <c r="D19" t="n">
+        <v>66.82821706567933</v>
+      </c>
+      <c r="E19" t="n">
+        <v>246.3768926558003</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>71.3408505026631</v>
+      </c>
+      <c r="C20" t="n">
+        <v>31.44400099216774</v>
+      </c>
+      <c r="D20" t="n">
+        <v>89.68396330689546</v>
+      </c>
+      <c r="E20" t="n">
+        <v>175.0206058959384</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>51.72019383735951</v>
+      </c>
+      <c r="C21" t="n">
+        <v>49.19410286708442</v>
+      </c>
+      <c r="D21" t="n">
+        <v>78.13301423822864</v>
+      </c>
+      <c r="E21" t="n">
+        <v>67.09870600284002</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>51.7186250379833</v>
+      </c>
+      <c r="C22" t="n">
+        <v>17.60015315178037</v>
+      </c>
+      <c r="D22" t="n">
+        <v>43.27340374137156</v>
+      </c>
+      <c r="E22" t="n">
+        <v>284.8391820244757</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>69.40936908332344</v>
+      </c>
+      <c r="C23" t="n">
+        <v>19.62893696133423</v>
+      </c>
+      <c r="D23" t="n">
+        <v>56.99976075483089</v>
+      </c>
+      <c r="E23" t="n">
+        <v>194.6874090543764</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>51.25308542623718</v>
+      </c>
+      <c r="C24" t="n">
+        <v>29.15207134664003</v>
+      </c>
+      <c r="D24" t="n">
+        <v>45.2883642559216</v>
+      </c>
+      <c r="E24" t="n">
+        <v>229.2857209557592</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>41.13036820845898</v>
+      </c>
+      <c r="C25" t="n">
+        <v>19.97382929730346</v>
+      </c>
+      <c r="D25" t="n">
+        <v>115.1827850933926</v>
+      </c>
+      <c r="E25" t="n">
+        <v>231.848824432004</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>42.93647957563869</v>
+      </c>
+      <c r="C26" t="n">
+        <v>94.81279528228055</v>
+      </c>
+      <c r="D26" t="n">
+        <v>60.96508497242434</v>
+      </c>
+      <c r="E26" t="n">
+        <v>280.9578742787604</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>